<commit_message>
Add management-informed scenario to LBO model
</commit_message>
<xml_diff>
--- a/excel/quinstreet_lbo.xlsx
+++ b/excel/quinstreet_lbo.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="177">
   <si>
     <t xml:space="preserve">QuinStreet LBO - purpose and method</t>
   </si>
@@ -234,21 +234,51 @@
     <t xml:space="preserve">Assumption: common PE return hurdle</t>
   </si>
   <si>
-    <t xml:space="preserve">Operating assumptions (FY2027-FY2031, base case)</t>
+    <t xml:space="preserve">Scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active scenario (1 = Ridgeline base case, 2 = management-informed case)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Choose which operating case drives the model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base case: revenue growth per year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption: organic growth well below the 30.6% CAGR, which was partly acquired</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Management-informed case: revenue growth per year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption: management guides ~16% for FY2027 (incl. a full year of HomeBuddy); assumed to fade, averaging 12%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base case: EBITDA margin reached in FY2031 (strict)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption: modest improvement from 4.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Management-informed case: EBITDA margin reached in FY2031 (strict)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption: FY2027 guidance (10.3% adjusted) implies ~6.3% strict after ~4 pts of add-backs; continued expansion to 8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operating assumptions (FY2027-FY2031), driven by the active scenario</t>
   </si>
   <si>
     <t xml:space="preserve">Revenue growth per year</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumption: organic growth well below the 30.6% CAGR, which was partly acquired</t>
+    <t xml:space="preserve">From the active scenario</t>
   </si>
   <si>
     <t xml:space="preserve">EBITDA margin reached in FY2031 (strict)</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumption: modest improvement from 4.7% (value-creation case)</t>
-  </si>
-  <si>
     <t xml:space="preserve">D&amp;A</t>
   </si>
   <si>
@@ -280,6 +310,9 @@
   </si>
   <si>
     <t xml:space="preserve">$ millions unless stated. Green = link to Inputs; black = formula. Every value traces to the Inputs sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active scenario:</t>
   </si>
   <si>
     <t xml:space="preserve">A. Purchase price</t>
@@ -536,7 +569,7 @@
     <numFmt numFmtId="170" formatCode="@"/>
     <numFmt numFmtId="171" formatCode="0.00\x"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -614,6 +647,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF008000"/>
       <name val="Arial"/>
@@ -697,7 +738,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -762,11 +803,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -774,7 +819,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -790,7 +835,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -818,7 +863,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -826,7 +871,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1191,7 +1236,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -1554,11 +1599,11 @@
       <c r="A33" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B33" s="11" t="n">
-        <v>0.08</v>
+      <c r="B33" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>72</v>
@@ -1568,8 +1613,8 @@
       <c r="A34" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B34" s="11" t="n">
-        <v>0.06</v>
+      <c r="B34" s="12" t="n">
+        <v>0.08</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>27</v>
@@ -1582,30 +1627,28 @@
       <c r="A35" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B35" s="15" t="n">
-        <f aca="false">B13/B11</f>
-        <v>0.0194790136816882</v>
+      <c r="B35" s="12" t="n">
+        <v>0.12</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B36" s="12" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="B36" s="15" t="n">
-        <f aca="false">(B15+B16)/B11</f>
-        <v>0.0110535672876246</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1613,27 +1656,109 @@
         <v>79</v>
       </c>
       <c r="B37" s="12" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B40" s="15" t="n">
+        <f aca="false">CHOOSE(B33,B34,B35)</f>
+        <v>0.08</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B41" s="15" t="n">
+        <f aca="false">CHOOSE(B33,B36,B37)</f>
+        <v>0.06</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B42" s="15" t="n">
+        <f aca="false">B13/B11</f>
+        <v>0.0194790136816882</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B43" s="15" t="n">
+        <f aca="false">(B15+B16)/B11</f>
+        <v>0.0110535672876246</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B44" s="12" t="n">
         <v>0.05</v>
       </c>
-      <c r="C37" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D37" s="2" t="s">
+      <c r="C44" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B38" s="14" t="n">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B45" s="14" t="n">
         <v>14.6</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>83</v>
+      <c r="C45" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1662,17 +1787,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>85</v>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" s="16" t="str">
+        <f aca="false">IF(Inputs!$B$33=1,"Ridgeline base case","Management-informed case")</f>
+        <v>Ridgeline base case</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -1684,133 +1818,133 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="16" t="n">
+        <v>98</v>
+      </c>
+      <c r="B5" s="17" t="n">
         <f aca="false">Inputs!$B$6</f>
         <v>16.52</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B6" s="17" t="n">
+        <v>99</v>
+      </c>
+      <c r="B6" s="18" t="n">
         <f aca="false">Inputs!$B$8</f>
         <v>0.3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B7" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="B7" s="19" t="n">
         <f aca="false">B5*(1+B6)</f>
         <v>21.476</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B8" s="19" t="n">
+        <v>101</v>
+      </c>
+      <c r="B8" s="20" t="n">
         <f aca="false">Inputs!$B$7</f>
         <v>57.1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B9" s="20" t="n">
+        <v>102</v>
+      </c>
+      <c r="B9" s="21" t="n">
         <f aca="false">B7*B8</f>
         <v>1226.2796</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B10" s="19" t="n">
+        <v>103</v>
+      </c>
+      <c r="B10" s="20" t="n">
         <f aca="false">Inputs!$B$18</f>
         <v>70</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B11" s="19" t="n">
+        <v>104</v>
+      </c>
+      <c r="B11" s="20" t="n">
         <f aca="false">Inputs!$B$17</f>
         <v>128.3</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B12" s="21" t="n">
+        <v>105</v>
+      </c>
+      <c r="B12" s="22" t="n">
         <f aca="false">B9+B10-B11</f>
         <v>1167.9796</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B13" s="19" t="n">
+        <v>106</v>
+      </c>
+      <c r="B13" s="20" t="n">
         <f aca="false">Inputs!$B$12</f>
         <v>60.6</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" s="22" t="n">
+        <v>107</v>
+      </c>
+      <c r="B14" s="23" t="n">
         <f aca="false">B12/B13</f>
         <v>19.2735907590759</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B15" s="20" t="n">
+        <v>108</v>
+      </c>
+      <c r="B15" s="21" t="n">
         <f aca="false">Inputs!$B$12+Inputs!$B$23*Inputs!$B$14</f>
         <v>98</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B16" s="22" t="n">
+        <v>109</v>
+      </c>
+      <c r="B16" s="23" t="n">
         <f aca="false">B12/B15</f>
         <v>11.9181591836735</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="B17" s="20" t="n">
+        <v>110</v>
+      </c>
+      <c r="B17" s="21" t="n">
         <f aca="false">B5*B8+B10-B11</f>
         <v>884.992</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B18" s="22" t="n">
+        <v>111</v>
+      </c>
+      <c r="B18" s="23" t="n">
         <f aca="false">B17/B13</f>
         <v>14.6038283828383</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -1821,24 +1955,24 @@
       <c r="H20" s="8"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
-        <v>102</v>
+      <c r="A21" s="24" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B22" s="20" t="n">
+        <v>114</v>
+      </c>
+      <c r="B22" s="21" t="n">
         <f aca="false">B9</f>
         <v>1226.2796</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="B23" s="20" t="n">
+        <v>115</v>
+      </c>
+      <c r="B23" s="21" t="n">
         <f aca="false">B10</f>
         <v>70</v>
       </c>
@@ -1847,30 +1981,30 @@
       <c r="A24" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="20" t="n">
+      <c r="B24" s="21" t="n">
         <f aca="false">B9*Inputs!$B$22</f>
         <v>36.788388</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B25" s="21" t="n">
+        <v>116</v>
+      </c>
+      <c r="B25" s="22" t="n">
         <f aca="false">SUM(B22:B24)</f>
         <v>1333.067988</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="23" t="s">
-        <v>106</v>
+      <c r="A26" s="24" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B27" s="20" t="n">
+        <v>118</v>
+      </c>
+      <c r="B27" s="21" t="n">
         <f aca="false">MAX(0,B11-Inputs!$B$21)</f>
         <v>98.3</v>
       </c>
@@ -1879,34 +2013,34 @@
       <c r="A28" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="20" t="n">
+      <c r="B28" s="21" t="n">
         <f aca="false">B15*Inputs!$B$24</f>
         <v>441</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="B29" s="24" t="n">
+        <v>119</v>
+      </c>
+      <c r="B29" s="25" t="n">
         <f aca="false">B25-B27-B28</f>
         <v>793.767988</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B30" s="21" t="n">
+        <v>120</v>
+      </c>
+      <c r="B30" s="22" t="n">
         <f aca="false">SUM(B27:B29)</f>
         <v>1333.067988</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B31" s="20" t="n">
+        <v>121</v>
+      </c>
+      <c r="B31" s="21" t="n">
         <f aca="false">B30-B25</f>
         <v>0</v>
       </c>
@@ -1915,32 +2049,32 @@
       <c r="A32" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="19" t="n">
+      <c r="B32" s="20" t="n">
         <f aca="false">Inputs!$B$29</f>
         <v>330</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="B33" s="25" t="str">
+        <v>122</v>
+      </c>
+      <c r="B33" s="26" t="str">
         <f aca="false">IF(B29&lt;=B32,"YES","NO")</f>
         <v>NO</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B34" s="22" t="n">
+        <v>123</v>
+      </c>
+      <c r="B34" s="23" t="n">
         <f aca="false">B28/B13</f>
         <v>7.27722772277228</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -1952,52 +2086,52 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B37" s="26"/>
-      <c r="C37" s="27" t="s">
-        <v>115</v>
-      </c>
-      <c r="D37" s="27" t="s">
-        <v>116</v>
-      </c>
-      <c r="E37" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="F37" s="27" t="s">
-        <v>118</v>
-      </c>
-      <c r="G37" s="27" t="s">
-        <v>119</v>
-      </c>
-      <c r="H37" s="27" t="s">
-        <v>120</v>
+        <v>125</v>
+      </c>
+      <c r="B37" s="27"/>
+      <c r="C37" s="28" t="s">
+        <v>126</v>
+      </c>
+      <c r="D37" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="E37" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="F37" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="G37" s="28" t="s">
+        <v>130</v>
+      </c>
+      <c r="H37" s="28" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>121</v>
-      </c>
-      <c r="C38" s="28" t="n">
+        <v>132</v>
+      </c>
+      <c r="C38" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="D38" s="29" t="n">
+      <c r="D38" s="30" t="n">
         <f aca="false">C38+1</f>
         <v>1</v>
       </c>
-      <c r="E38" s="29" t="n">
+      <c r="E38" s="30" t="n">
         <f aca="false">D38+1</f>
         <v>2</v>
       </c>
-      <c r="F38" s="29" t="n">
+      <c r="F38" s="30" t="n">
         <f aca="false">E38+1</f>
         <v>3</v>
       </c>
-      <c r="G38" s="29" t="n">
+      <c r="G38" s="30" t="n">
         <f aca="false">F38+1</f>
         <v>4</v>
       </c>
-      <c r="H38" s="29" t="n">
+      <c r="H38" s="30" t="n">
         <f aca="false">G38+1</f>
         <v>5</v>
       </c>
@@ -2006,34 +2140,34 @@
       <c r="A39" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C39" s="19" t="n">
+      <c r="C39" s="20" t="n">
         <f aca="false">Inputs!$B$11</f>
         <v>1293.7</v>
       </c>
-      <c r="D39" s="20" t="n">
-        <f aca="false">C39*(1+Inputs!$B$33)</f>
+      <c r="D39" s="21" t="n">
+        <f aca="false">C39*(1+Inputs!$B$40)</f>
         <v>1397.196</v>
       </c>
-      <c r="E39" s="20" t="n">
-        <f aca="false">D39*(1+Inputs!$B$33)</f>
+      <c r="E39" s="21" t="n">
+        <f aca="false">D39*(1+Inputs!$B$40)</f>
         <v>1508.97168</v>
       </c>
-      <c r="F39" s="20" t="n">
-        <f aca="false">E39*(1+Inputs!$B$33)</f>
+      <c r="F39" s="21" t="n">
+        <f aca="false">E39*(1+Inputs!$B$40)</f>
         <v>1629.6894144</v>
       </c>
-      <c r="G39" s="20" t="n">
-        <f aca="false">F39*(1+Inputs!$B$33)</f>
+      <c r="G39" s="21" t="n">
+        <f aca="false">F39*(1+Inputs!$B$40)</f>
         <v>1760.064567552</v>
       </c>
-      <c r="H39" s="20" t="n">
-        <f aca="false">G39*(1+Inputs!$B$33)</f>
+      <c r="H39" s="21" t="n">
+        <f aca="false">G39*(1+Inputs!$B$40)</f>
         <v>1900.86973295616</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="D40" s="15" t="n">
         <f aca="false">D39/C39-1</f>
@@ -2058,58 +2192,58 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C41" s="15" t="n">
         <f aca="false">C42/C39</f>
         <v>0.0468423900440597</v>
       </c>
       <c r="D41" s="15" t="n">
-        <f aca="false">$C$41+(Inputs!$B$34-$C$41)*D38/$H$38</f>
+        <f aca="false">$C$41+(Inputs!$B$41-$C$41)*D38/$H$38</f>
         <v>0.0494739120352477</v>
       </c>
       <c r="E41" s="15" t="n">
-        <f aca="false">$C$41+(Inputs!$B$34-$C$41)*E38/$H$38</f>
+        <f aca="false">$C$41+(Inputs!$B$41-$C$41)*E38/$H$38</f>
         <v>0.0521054340264358</v>
       </c>
       <c r="F41" s="15" t="n">
-        <f aca="false">$C$41+(Inputs!$B$34-$C$41)*F38/$H$38</f>
+        <f aca="false">$C$41+(Inputs!$B$41-$C$41)*F38/$H$38</f>
         <v>0.0547369560176239</v>
       </c>
       <c r="G41" s="15" t="n">
-        <f aca="false">$C$41+(Inputs!$B$34-$C$41)*G38/$H$38</f>
+        <f aca="false">$C$41+(Inputs!$B$41-$C$41)*G38/$H$38</f>
         <v>0.0573684780088119</v>
       </c>
       <c r="H41" s="15" t="n">
-        <f aca="false">$C$41+(Inputs!$B$34-$C$41)*H38/$H$38</f>
+        <f aca="false">$C$41+(Inputs!$B$41-$C$41)*H38/$H$38</f>
         <v>0.06</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C42" s="30" t="n">
+        <v>135</v>
+      </c>
+      <c r="C42" s="31" t="n">
         <f aca="false">Inputs!$B$12</f>
         <v>60.6</v>
       </c>
-      <c r="D42" s="21" t="n">
+      <c r="D42" s="22" t="n">
         <f aca="false">D39*D41</f>
         <v>69.124752</v>
       </c>
-      <c r="E42" s="21" t="n">
+      <c r="E42" s="22" t="n">
         <f aca="false">E39*E41</f>
         <v>78.62562432</v>
       </c>
-      <c r="F42" s="21" t="n">
+      <c r="F42" s="22" t="n">
         <f aca="false">F39*F41</f>
         <v>89.2042377984</v>
       </c>
-      <c r="G42" s="21" t="n">
+      <c r="G42" s="22" t="n">
         <f aca="false">G39*G41</f>
         <v>100.972225437696</v>
       </c>
-      <c r="H42" s="21" t="n">
+      <c r="H42" s="22" t="n">
         <f aca="false">H39*H41</f>
         <v>114.05218397737</v>
       </c>
@@ -2118,218 +2252,218 @@
       <c r="A43" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C43" s="19" t="n">
+      <c r="C43" s="20" t="n">
         <f aca="false">Inputs!$B$13</f>
         <v>25.2</v>
       </c>
-      <c r="D43" s="20" t="n">
-        <f aca="false">D39*Inputs!$B$35</f>
+      <c r="D43" s="21" t="n">
+        <f aca="false">D39*Inputs!$B$42</f>
         <v>27.216</v>
       </c>
-      <c r="E43" s="20" t="n">
-        <f aca="false">E39*Inputs!$B$35</f>
+      <c r="E43" s="21" t="n">
+        <f aca="false">E39*Inputs!$B$42</f>
         <v>29.39328</v>
       </c>
-      <c r="F43" s="20" t="n">
-        <f aca="false">F39*Inputs!$B$35</f>
+      <c r="F43" s="21" t="n">
+        <f aca="false">F39*Inputs!$B$42</f>
         <v>31.7447424</v>
       </c>
-      <c r="G43" s="20" t="n">
-        <f aca="false">G39*Inputs!$B$35</f>
+      <c r="G43" s="21" t="n">
+        <f aca="false">G39*Inputs!$B$42</f>
         <v>34.284321792</v>
       </c>
-      <c r="H43" s="20" t="n">
-        <f aca="false">H39*Inputs!$B$35</f>
+      <c r="H43" s="21" t="n">
+        <f aca="false">H39*Inputs!$B$42</f>
         <v>37.02706753536</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C44" s="20" t="n">
+        <v>136</v>
+      </c>
+      <c r="C44" s="21" t="n">
         <f aca="false">C42-C43</f>
         <v>35.4</v>
       </c>
-      <c r="D44" s="20" t="n">
+      <c r="D44" s="21" t="n">
         <f aca="false">D42-D43</f>
         <v>41.908752</v>
       </c>
-      <c r="E44" s="20" t="n">
+      <c r="E44" s="21" t="n">
         <f aca="false">E42-E43</f>
         <v>49.23234432</v>
       </c>
-      <c r="F44" s="20" t="n">
+      <c r="F44" s="21" t="n">
         <f aca="false">F42-F43</f>
         <v>57.4594953984</v>
       </c>
-      <c r="G44" s="20" t="n">
+      <c r="G44" s="21" t="n">
         <f aca="false">G42-G43</f>
         <v>66.687903645696</v>
       </c>
-      <c r="H44" s="20" t="n">
+      <c r="H44" s="21" t="n">
         <f aca="false">H42-H43</f>
         <v>77.0251164420096</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="D45" s="20" t="n">
+        <v>137</v>
+      </c>
+      <c r="D45" s="21" t="n">
         <f aca="false">D53*Inputs!$B$25</f>
         <v>37.485</v>
       </c>
-      <c r="E45" s="20" t="n">
+      <c r="E45" s="21" t="n">
         <f aca="false">E53*Inputs!$B$25</f>
         <v>36.64222381</v>
       </c>
-      <c r="F45" s="20" t="n">
+      <c r="F45" s="21" t="n">
         <f aca="false">F53*Inputs!$B$25</f>
         <v>35.2339806674875</v>
       </c>
-      <c r="G45" s="20" t="n">
+      <c r="G45" s="21" t="n">
         <f aca="false">G53*Inputs!$B$25</f>
         <v>33.1630313065918</v>
       </c>
-      <c r="H45" s="20" t="n">
+      <c r="H45" s="21" t="n">
         <f aca="false">H53*Inputs!$B$25</f>
         <v>30.3194220744299</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="D46" s="20" t="n">
+        <v>138</v>
+      </c>
+      <c r="D46" s="21" t="n">
         <f aca="false">D44-D45</f>
         <v>4.42375199999999</v>
       </c>
-      <c r="E46" s="20" t="n">
+      <c r="E46" s="21" t="n">
         <f aca="false">E44-E45</f>
         <v>12.59012051</v>
       </c>
-      <c r="F46" s="20" t="n">
+      <c r="F46" s="21" t="n">
         <f aca="false">F44-F45</f>
         <v>22.2255147309125</v>
       </c>
-      <c r="G46" s="20" t="n">
+      <c r="G46" s="21" t="n">
         <f aca="false">G44-G45</f>
         <v>33.5248723391042</v>
       </c>
-      <c r="H46" s="20" t="n">
+      <c r="H46" s="21" t="n">
         <f aca="false">H44-H45</f>
         <v>46.7056943675797</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="D47" s="20" t="n">
+        <v>139</v>
+      </c>
+      <c r="D47" s="21" t="n">
         <f aca="false">MAX(0,D46)*Inputs!$B$28</f>
         <v>1.105938</v>
       </c>
-      <c r="E47" s="20" t="n">
+      <c r="E47" s="21" t="n">
         <f aca="false">MAX(0,E46)*Inputs!$B$28</f>
         <v>3.1475301275</v>
       </c>
-      <c r="F47" s="20" t="n">
+      <c r="F47" s="21" t="n">
         <f aca="false">MAX(0,F46)*Inputs!$B$28</f>
         <v>5.55637868272813</v>
       </c>
-      <c r="G47" s="20" t="n">
+      <c r="G47" s="21" t="n">
         <f aca="false">MAX(0,G46)*Inputs!$B$28</f>
         <v>8.38121808477605</v>
       </c>
-      <c r="H47" s="20" t="n">
+      <c r="H47" s="21" t="n">
         <f aca="false">MAX(0,H46)*Inputs!$B$28</f>
         <v>11.6764235918949</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C48" s="19" t="n">
+        <v>88</v>
+      </c>
+      <c r="C48" s="20" t="n">
         <f aca="false">Inputs!$B$15+Inputs!$B$16</f>
         <v>14.3</v>
       </c>
-      <c r="D48" s="20" t="n">
-        <f aca="false">D39*Inputs!$B$36</f>
+      <c r="D48" s="21" t="n">
+        <f aca="false">D39*Inputs!$B$43</f>
         <v>15.444</v>
       </c>
-      <c r="E48" s="20" t="n">
-        <f aca="false">E39*Inputs!$B$36</f>
+      <c r="E48" s="21" t="n">
+        <f aca="false">E39*Inputs!$B$43</f>
         <v>16.67952</v>
       </c>
-      <c r="F48" s="20" t="n">
-        <f aca="false">F39*Inputs!$B$36</f>
+      <c r="F48" s="21" t="n">
+        <f aca="false">F39*Inputs!$B$43</f>
         <v>18.0138816</v>
       </c>
-      <c r="G48" s="20" t="n">
-        <f aca="false">G39*Inputs!$B$36</f>
+      <c r="G48" s="21" t="n">
+        <f aca="false">G39*Inputs!$B$43</f>
         <v>19.454992128</v>
       </c>
-      <c r="H48" s="20" t="n">
-        <f aca="false">H39*Inputs!$B$36</f>
+      <c r="H48" s="21" t="n">
+        <f aca="false">H39*Inputs!$B$43</f>
         <v>21.01139149824</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="D49" s="20" t="n">
-        <f aca="false">(D39-C39)*Inputs!$B$37</f>
+        <v>140</v>
+      </c>
+      <c r="D49" s="21" t="n">
+        <f aca="false">(D39-C39)*Inputs!$B$44</f>
         <v>5.17480000000001</v>
       </c>
-      <c r="E49" s="20" t="n">
-        <f aca="false">(E39-D39)*Inputs!$B$37</f>
+      <c r="E49" s="21" t="n">
+        <f aca="false">(E39-D39)*Inputs!$B$44</f>
         <v>5.58878400000001</v>
       </c>
-      <c r="F49" s="20" t="n">
-        <f aca="false">(F39-E39)*Inputs!$B$37</f>
+      <c r="F49" s="21" t="n">
+        <f aca="false">(F39-E39)*Inputs!$B$44</f>
         <v>6.03588672000001</v>
       </c>
-      <c r="G49" s="20" t="n">
-        <f aca="false">(G39-F39)*Inputs!$B$37</f>
+      <c r="G49" s="21" t="n">
+        <f aca="false">(G39-F39)*Inputs!$B$44</f>
         <v>6.51875765760001</v>
       </c>
-      <c r="H49" s="20" t="n">
-        <f aca="false">(H39-G39)*Inputs!$B$37</f>
+      <c r="H49" s="21" t="n">
+        <f aca="false">(H39-G39)*Inputs!$B$44</f>
         <v>7.04025827020801</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C50" s="31"/>
-      <c r="D50" s="21" t="n">
+        <v>141</v>
+      </c>
+      <c r="C50" s="32"/>
+      <c r="D50" s="22" t="n">
         <f aca="false">D42-D47-D48-D49-D45</f>
         <v>9.915014</v>
       </c>
-      <c r="E50" s="21" t="n">
+      <c r="E50" s="22" t="n">
         <f aca="false">E42-E47-E48-E49-E45</f>
         <v>16.5675663825</v>
       </c>
-      <c r="F50" s="21" t="n">
+      <c r="F50" s="22" t="n">
         <f aca="false">F42-F47-F48-F49-F45</f>
         <v>24.3641101281844</v>
       </c>
-      <c r="G50" s="21" t="n">
+      <c r="G50" s="22" t="n">
         <f aca="false">G42-G47-G48-G49-G45</f>
         <v>33.4542262607281</v>
       </c>
-      <c r="H50" s="21" t="n">
+      <c r="H50" s="22" t="n">
         <f aca="false">H42-H47-H48-H49-H45</f>
         <v>44.0046885425968</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
@@ -2341,25 +2475,25 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D53" s="20" t="n">
+        <v>143</v>
+      </c>
+      <c r="D53" s="21" t="n">
         <f aca="false">C56</f>
         <v>441</v>
       </c>
-      <c r="E53" s="20" t="n">
+      <c r="E53" s="21" t="n">
         <f aca="false">D56</f>
         <v>431.084986</v>
       </c>
-      <c r="F53" s="20" t="n">
+      <c r="F53" s="21" t="n">
         <f aca="false">E56</f>
         <v>414.5174196175</v>
       </c>
-      <c r="G53" s="20" t="n">
+      <c r="G53" s="21" t="n">
         <f aca="false">F56</f>
         <v>390.153309489316</v>
       </c>
-      <c r="H53" s="20" t="n">
+      <c r="H53" s="21" t="n">
         <f aca="false">G56</f>
         <v>356.699083228587</v>
       </c>
@@ -2368,196 +2502,196 @@
       <c r="A54" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D54" s="20" t="n">
+      <c r="D54" s="21" t="n">
         <f aca="false">MIN(D53,$B$28*Inputs!$B$26)</f>
         <v>4.41</v>
       </c>
-      <c r="E54" s="20" t="n">
+      <c r="E54" s="21" t="n">
         <f aca="false">MIN(E53,$B$28*Inputs!$B$26)</f>
         <v>4.41</v>
       </c>
-      <c r="F54" s="20" t="n">
+      <c r="F54" s="21" t="n">
         <f aca="false">MIN(F53,$B$28*Inputs!$B$26)</f>
         <v>4.41</v>
       </c>
-      <c r="G54" s="20" t="n">
+      <c r="G54" s="21" t="n">
         <f aca="false">MIN(G53,$B$28*Inputs!$B$26)</f>
         <v>4.41</v>
       </c>
-      <c r="H54" s="20" t="n">
+      <c r="H54" s="21" t="n">
         <f aca="false">MIN(H53,$B$28*Inputs!$B$26)</f>
         <v>4.41</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D55" s="20" t="n">
+        <v>144</v>
+      </c>
+      <c r="D55" s="21" t="n">
         <f aca="false">MIN(D53-D54,MAX(0,D50-D54)*Inputs!$B$27)</f>
         <v>5.505014</v>
       </c>
-      <c r="E55" s="20" t="n">
+      <c r="E55" s="21" t="n">
         <f aca="false">MIN(E53-E54,MAX(0,E50-E54)*Inputs!$B$27)</f>
         <v>12.1575663825</v>
       </c>
-      <c r="F55" s="20" t="n">
+      <c r="F55" s="21" t="n">
         <f aca="false">MIN(F53-F54,MAX(0,F50-F54)*Inputs!$B$27)</f>
         <v>19.9541101281844</v>
       </c>
-      <c r="G55" s="20" t="n">
+      <c r="G55" s="21" t="n">
         <f aca="false">MIN(G53-G54,MAX(0,G50-G54)*Inputs!$B$27)</f>
         <v>29.0442262607281</v>
       </c>
-      <c r="H55" s="20" t="n">
+      <c r="H55" s="21" t="n">
         <f aca="false">MIN(H53-H54,MAX(0,H50-H54)*Inputs!$B$27)</f>
         <v>39.5946885425968</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C56" s="21" t="n">
+        <v>145</v>
+      </c>
+      <c r="C56" s="22" t="n">
         <f aca="false">B28</f>
         <v>441</v>
       </c>
-      <c r="D56" s="21" t="n">
+      <c r="D56" s="22" t="n">
         <f aca="false">D53-D54-D55</f>
         <v>431.084986</v>
       </c>
-      <c r="E56" s="21" t="n">
+      <c r="E56" s="22" t="n">
         <f aca="false">E53-E54-E55</f>
         <v>414.5174196175</v>
       </c>
-      <c r="F56" s="21" t="n">
+      <c r="F56" s="22" t="n">
         <f aca="false">F53-F54-F55</f>
         <v>390.153309489316</v>
       </c>
-      <c r="G56" s="21" t="n">
+      <c r="G56" s="22" t="n">
         <f aca="false">G53-G54-G55</f>
         <v>356.699083228587</v>
       </c>
-      <c r="H56" s="21" t="n">
+      <c r="H56" s="22" t="n">
         <f aca="false">H53-H54-H55</f>
         <v>312.694394685991</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="D57" s="20" t="n">
+        <v>146</v>
+      </c>
+      <c r="D57" s="21" t="n">
         <f aca="false">C58</f>
         <v>30</v>
       </c>
-      <c r="E57" s="20" t="n">
+      <c r="E57" s="21" t="n">
         <f aca="false">D58</f>
         <v>30</v>
       </c>
-      <c r="F57" s="20" t="n">
+      <c r="F57" s="21" t="n">
         <f aca="false">E58</f>
         <v>30</v>
       </c>
-      <c r="G57" s="20" t="n">
+      <c r="G57" s="21" t="n">
         <f aca="false">F58</f>
         <v>30</v>
       </c>
-      <c r="H57" s="20" t="n">
+      <c r="H57" s="21" t="n">
         <f aca="false">G58</f>
         <v>30</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="C58" s="19" t="n">
+        <v>147</v>
+      </c>
+      <c r="C58" s="20" t="n">
         <f aca="false">Inputs!$B$21</f>
         <v>30</v>
       </c>
-      <c r="D58" s="20" t="n">
+      <c r="D58" s="21" t="n">
         <f aca="false">D57+D50-D54-D55</f>
         <v>30</v>
       </c>
-      <c r="E58" s="20" t="n">
+      <c r="E58" s="21" t="n">
         <f aca="false">E57+E50-E54-E55</f>
         <v>30</v>
       </c>
-      <c r="F58" s="20" t="n">
+      <c r="F58" s="21" t="n">
         <f aca="false">F57+F50-F54-F55</f>
         <v>30</v>
       </c>
-      <c r="G58" s="20" t="n">
+      <c r="G58" s="21" t="n">
         <f aca="false">G57+G50-G54-G55</f>
         <v>30</v>
       </c>
-      <c r="H58" s="20" t="n">
+      <c r="H58" s="21" t="n">
         <f aca="false">H57+H50-H54-H55</f>
         <v>30</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C59" s="24" t="n">
+        <v>148</v>
+      </c>
+      <c r="C59" s="25" t="n">
         <f aca="false">C56-C58</f>
         <v>411</v>
       </c>
-      <c r="D59" s="24" t="n">
+      <c r="D59" s="25" t="n">
         <f aca="false">D56-D58</f>
         <v>401.084986</v>
       </c>
-      <c r="E59" s="24" t="n">
+      <c r="E59" s="25" t="n">
         <f aca="false">E56-E58</f>
         <v>384.5174196175</v>
       </c>
-      <c r="F59" s="24" t="n">
+      <c r="F59" s="25" t="n">
         <f aca="false">F56-F58</f>
         <v>360.153309489316</v>
       </c>
-      <c r="G59" s="24" t="n">
+      <c r="G59" s="25" t="n">
         <f aca="false">G56-G58</f>
         <v>326.699083228587</v>
       </c>
-      <c r="H59" s="24" t="n">
+      <c r="H59" s="25" t="n">
         <f aca="false">H56-H58</f>
         <v>282.694394685991</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C60" s="22" t="n">
+        <v>149</v>
+      </c>
+      <c r="C60" s="23" t="n">
         <f aca="false">C59/C42</f>
         <v>6.78217821782178</v>
       </c>
-      <c r="D60" s="22" t="n">
+      <c r="D60" s="23" t="n">
         <f aca="false">D59/D42</f>
         <v>5.80233526190445</v>
       </c>
-      <c r="E60" s="22" t="n">
+      <c r="E60" s="23" t="n">
         <f aca="false">E59/E42</f>
         <v>4.89048478715469</v>
       </c>
-      <c r="F60" s="22" t="n">
+      <c r="F60" s="23" t="n">
         <f aca="false">F59/F42</f>
         <v>4.03740134300856</v>
       </c>
-      <c r="G60" s="22" t="n">
+      <c r="G60" s="23" t="n">
         <f aca="false">G59/G42</f>
         <v>3.23553414627049</v>
       </c>
-      <c r="H60" s="22" t="n">
+      <c r="H60" s="23" t="n">
         <f aca="false">H59/H42</f>
         <v>2.4786407837844</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="8"/>
@@ -2569,81 +2703,81 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="B63" s="20" t="n">
+        <v>151</v>
+      </c>
+      <c r="B63" s="21" t="n">
         <f aca="false">H42</f>
         <v>114.05218397737</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="B64" s="32" t="n">
-        <f aca="false">Inputs!$B$38</f>
+        <v>152</v>
+      </c>
+      <c r="B64" s="33" t="n">
+        <f aca="false">Inputs!$B$45</f>
         <v>14.6</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="B65" s="20" t="n">
+        <v>153</v>
+      </c>
+      <c r="B65" s="21" t="n">
         <f aca="false">B63*B64</f>
         <v>1665.1618860696</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="B66" s="20" t="n">
+        <v>154</v>
+      </c>
+      <c r="B66" s="21" t="n">
         <f aca="false">H56</f>
         <v>312.694394685991</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="B67" s="20" t="n">
+        <v>155</v>
+      </c>
+      <c r="B67" s="21" t="n">
         <f aca="false">H58</f>
         <v>30</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B68" s="21" t="n">
+        <v>156</v>
+      </c>
+      <c r="B68" s="22" t="n">
         <f aca="false">B65-B66+B67</f>
         <v>1382.46749138361</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="B69" s="20" t="n">
+        <v>157</v>
+      </c>
+      <c r="B69" s="21" t="n">
         <f aca="false">B29</f>
         <v>793.767988</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="B70" s="33" t="n">
+        <v>158</v>
+      </c>
+      <c r="B70" s="34" t="n">
         <f aca="false">B68/B69</f>
         <v>1.74165185833068</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B71" s="34" t="n">
+        <v>159</v>
+      </c>
+      <c r="B71" s="35" t="n">
         <f aca="false">B70^(1/H38)-1</f>
         <v>0.117357811468411</v>
       </c>
@@ -2652,23 +2786,23 @@
       <c r="A72" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B72" s="17" t="n">
+      <c r="B72" s="18" t="n">
         <f aca="false">Inputs!$B$30</f>
         <v>0.2</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="B73" s="25" t="str">
+        <v>160</v>
+      </c>
+      <c r="B73" s="26" t="str">
         <f aca="false">IF(B71&gt;=B72,"YES","NO")</f>
         <v>NO</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="B75" s="8"/>
       <c r="C75" s="8"/>
@@ -2680,70 +2814,70 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B76" s="22" t="n">
+        <v>107</v>
+      </c>
+      <c r="B76" s="23" t="n">
         <f aca="false">B14</f>
         <v>19.2735907590759</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="B77" s="20" t="n">
+        <v>162</v>
+      </c>
+      <c r="B77" s="21" t="n">
         <f aca="false">(B63-B13)*B76</f>
         <v>1030.21551915866</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="B78" s="20" t="n">
+        <v>163</v>
+      </c>
+      <c r="B78" s="21" t="n">
         <f aca="false">(B64-B76)*B63</f>
         <v>-533.03323308906</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B79" s="20" t="n">
+        <v>164</v>
+      </c>
+      <c r="B79" s="21" t="n">
         <f aca="false">C59-H59</f>
         <v>128.305605314009</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B80" s="20" t="n">
+        <v>165</v>
+      </c>
+      <c r="B80" s="21" t="n">
         <f aca="false">-B24</f>
         <v>-36.788388</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B81" s="21" t="n">
+        <v>166</v>
+      </c>
+      <c r="B81" s="22" t="n">
         <f aca="false">SUM(B77:B80)</f>
         <v>588.699503383606</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="B82" s="20" t="n">
+        <v>167</v>
+      </c>
+      <c r="B82" s="21" t="n">
         <f aca="false">B81-(B68-B69)</f>
         <v>0</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="B84" s="8"/>
       <c r="C84" s="8"/>
@@ -2755,70 +2889,70 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="B85" s="20" t="n">
+        <v>169</v>
+      </c>
+      <c r="B85" s="21" t="n">
         <f aca="false">B68/(1+B72)^H38</f>
         <v>555.582678828931</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="B86" s="18" t="n">
+        <v>170</v>
+      </c>
+      <c r="B86" s="19" t="n">
         <f aca="false">(B85+B27+B28-B23)/(1+Inputs!$B$22)/B8</f>
         <v>17.426124816434</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="B87" s="18" t="n">
+        <v>171</v>
+      </c>
+      <c r="B87" s="19" t="n">
         <f aca="false">(B32+B27+B28-B23)/(1+Inputs!$B$22)/B8</f>
         <v>13.5905327053543</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="B88" s="35" t="n">
+        <v>172</v>
+      </c>
+      <c r="B88" s="36" t="n">
         <f aca="false">MIN(B86,B87)</f>
         <v>13.5905327053543</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="B89" s="36" t="str">
+        <v>173</v>
+      </c>
+      <c r="B89" s="37" t="str">
         <f aca="false">IF(B86&lt;B87,"Target IRR","Equity limit")</f>
         <v>Equity limit</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="B90" s="34" t="n">
+        <v>174</v>
+      </c>
+      <c r="B90" s="35" t="n">
         <f aca="false">B88/B5-1</f>
         <v>-0.177328528731582</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="B91" s="25" t="str">
+        <v>175</v>
+      </c>
+      <c r="B91" s="26" t="str">
         <f aca="false">IF(B88&lt;B5,"PASS: cannot pay even the current market price",IF(B88&lt;B5*1.2,"MARGINAL: below a typical 20%+ takeover premium","ACTIONABLE: can pay a competitive premium"))</f>
         <v>PASS: cannot pay even the current market price</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="5" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>